<commit_message>
FIX: Update data files and code across multiple papers
</commit_message>
<xml_diff>
--- a/Task Update.xlsx
+++ b/Task Update.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Data\CS-P4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\CS-P4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08FA758B-0405-4992-987C-D2B185DA8736}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{022FE4BE-07D7-487C-BF6B-4767BB826AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="26">
   <si>
     <t>S.No.</t>
   </si>
@@ -88,6 +88,21 @@
   </si>
   <si>
     <t>9618_s24_42</t>
+  </si>
+  <si>
+    <t>Q1 by SuhairPasta</t>
+  </si>
+  <si>
+    <t>Completed By AmmarSAA</t>
+  </si>
+  <si>
+    <t>9618_w23_42</t>
+  </si>
+  <si>
+    <t>9618_s23_42</t>
+  </si>
+  <si>
+    <t>9618_w24_42</t>
   </si>
 </sst>
 </file>
@@ -474,7 +489,7 @@
         <v>6</v>
       </c>
       <c r="F2" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -498,9 +513,12 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -509,7 +527,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -517,7 +541,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -525,13 +549,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -539,12 +557,12 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" t="s">
         <v>15</v>
       </c>
     </row>
@@ -553,9 +571,12 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C10" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s">
         <v>15</v>
       </c>
     </row>
@@ -564,10 +585,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -575,10 +596,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -586,27 +607,45 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
-      </c>
-      <c r="D13" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
FEAT: 9618_s21_42 questions, update .gitignore and Task Update
</commit_message>
<xml_diff>
--- a/Task Update.xlsx
+++ b/Task Update.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data\CS-P4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CS-P4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{022FE4BE-07D7-487C-BF6B-4767BB826AC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F92D1A82-27C8-4F66-A163-5765BC20D39C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="26">
   <si>
     <t>S.No.</t>
   </si>
@@ -499,6 +499,18 @@
       <c r="B3" t="s">
         <v>17</v>
       </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">

</xml_diff>